<commit_message>
Setup the projects present in month
</commit_message>
<xml_diff>
--- a/TimesheetFs/Timesheet-Template-v10.xlsx
+++ b/TimesheetFs/Timesheet-Template-v10.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Perso\Taggl\TimesheetFs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A99E397B-090B-4860-AE0D-44576CB3A6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB2AFD74-C5A9-4105-B56B-4C7CA5F79E10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{FB794F17-9F1B-438B-B219-D10D95E788D4}"/>
+    <workbookView xWindow="7485" yWindow="4920" windowWidth="28800" windowHeight="15105" activeTab="1" xr2:uid="{FB794F17-9F1B-438B-B219-D10D95E788D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="5" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="147">
   <si>
     <t>Code</t>
   </si>
@@ -763,9 +763,6 @@
   </si>
   <si>
     <t>Wavenet</t>
-  </si>
-  <si>
-    <t>OffresInsertion</t>
   </si>
 </sst>
 </file>
@@ -3502,12 +3499,10 @@
       <c r="AI6" s="2"/>
     </row>
     <row r="7" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B7" s="41" t="s">
-        <v>112</v>
-      </c>
+      <c r="B7" s="41"/>
       <c r="C7" s="42" t="str">
         <f>IF(ISBLANK(B7),"",VLOOKUP(B7,'Codes projet'!$A$2:$B$801,2,FALSE))</f>
-        <v>Back Office HRXML</v>
+        <v/>
       </c>
       <c r="D7" s="50"/>
       <c r="E7" s="51"/>
@@ -3542,12 +3537,10 @@
       <c r="AH7" s="52"/>
     </row>
     <row r="8" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B8" s="43" t="s">
-        <v>52</v>
-      </c>
+      <c r="B8" s="43"/>
       <c r="C8" s="44" t="str">
         <f>IF(ISBLANK(B8),"",VLOOKUP(B8,'Codes projet'!$A$2:$B$801,2,FALSE))</f>
-        <v>CRM</v>
+        <v/>
       </c>
       <c r="D8" s="53"/>
       <c r="E8" s="54"/>
@@ -3582,12 +3575,10 @@
       <c r="AH8" s="55"/>
     </row>
     <row r="9" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B9" s="43" t="s">
-        <v>44</v>
-      </c>
+      <c r="B9" s="43"/>
       <c r="C9" s="44" t="str">
         <f>IF(ISBLANK(B9),"",VLOOKUP(B9,'Codes projet'!$A$2:$B$801,2,FALSE))</f>
-        <v>Dossier unique - Employeur</v>
+        <v/>
       </c>
       <c r="D9" s="53"/>
       <c r="E9" s="54"/>
@@ -3622,11 +3613,10 @@
       <c r="AH9" s="55"/>
     </row>
     <row r="10" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B10" s="43" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>147</v>
+      <c r="B10" s="43"/>
+      <c r="C10" s="44" t="str">
+        <f>IF(ISBLANK(B10),"",VLOOKUP(B10,'Codes projet'!$A$2:$B$801,2,FALSE))</f>
+        <v/>
       </c>
       <c r="D10" s="53"/>
       <c r="E10" s="54"/>
@@ -7786,11 +7776,11 @@
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="104" t="str">
         <f>IF(ISBLANK(Prestations!B7),"",Prestations!B7)</f>
-        <v>BOHRXML</v>
+        <v/>
       </c>
       <c r="C13" s="168" t="str">
         <f>Prestations!C7</f>
-        <v>Back Office HRXML</v>
+        <v/>
       </c>
       <c r="D13" s="169"/>
       <c r="E13" s="105" t="str">
@@ -7817,11 +7807,11 @@
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B8),"",Prestations!B8)</f>
-        <v>C107-01</v>
+        <v/>
       </c>
       <c r="C14" s="158" t="str">
         <f>Prestations!C8</f>
-        <v>CRM</v>
+        <v/>
       </c>
       <c r="D14" s="159"/>
       <c r="E14" s="108" t="str">
@@ -7848,11 +7838,11 @@
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B9),"",Prestations!B9)</f>
-        <v>C032-02</v>
+        <v/>
       </c>
       <c r="C15" s="158" t="str">
         <f>Prestations!C9</f>
-        <v>Dossier unique - Employeur</v>
+        <v/>
       </c>
       <c r="D15" s="159"/>
       <c r="E15" s="108" t="str">
@@ -7879,11 +7869,11 @@
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B10),"",Prestations!B10)</f>
-        <v>AUTRE</v>
+        <v/>
       </c>
       <c r="C16" s="158" t="str">
         <f>Prestations!C10</f>
-        <v>OffresInsertion</v>
+        <v/>
       </c>
       <c r="D16" s="159"/>
       <c r="E16" s="108" t="str">

</xml_diff>